<commit_message>
Add a required_deity column for archetypes
New Archetypes sheet column required_deity lists the deities an
archetype needs (comma-separated, as on the Deities sheet). Midnight
Illusionist requires Zon-Kuthon. Only cells M1 and M133 were added.

A locked deity limits the archetype roll to archetypes that accept it.
Otherwise the archetype needs one of its deities to pass the source and
access filters, and then sets the deity from its list, even with deity
rolling off. A locked archetype with an unmet deity requirement is
reported by findLockConflict, and archetype error messages now list the
requirements.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/data/generatordata.xlsx
+++ b/assets/data/generatordata.xlsx
@@ -28105,7 +28105,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A88DAEB-E71A-418F-A6F0-324150077FCF}">
-  <dimension ref="A1:L231"/>
+  <dimension ref="A1:M231"/>
   <sheetFormatPr defaultColWidth="80" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
@@ -28122,7 +28122,7 @@
     <col min="12" max="12" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -28158,6 +28158,11 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>1047</v>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>required_deity</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -31116,7 +31121,7 @@
       <c r="K132" s="2"/>
       <c r="L132" s="2"/>
     </row>
-    <row r="133" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>2231</v>
       </c>
@@ -31141,6 +31146,11 @@
       <c r="J133" s="2"/>
       <c r="K133" s="2"/>
       <c r="L133" s="2"/>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>Zon-Kuthon</t>
+        </is>
+      </c>
     </row>
     <row r="134" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">

</xml_diff>